<commit_message>
Procurement Dashboard KPI Changes Upto 8
Changes up to 8th KPI
</commit_message>
<xml_diff>
--- a/IntelliSource Dashboard KPI Changes.xlsx
+++ b/IntelliSource Dashboard KPI Changes.xlsx
@@ -1,13 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aryan\OneDrive\Documents\GitHub\kpmg-intelliflow\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAD905E0-6413-4F8A-8B6A-0B3327B09207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Procurement Dashboard KPIs" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,9 +24,323 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="57">
+  <si>
+    <t>Procurement Dashboard — KPIs</t>
+  </si>
+  <si>
+    <t>Target user: Procurement Managers | Refresh: Weekly | Purpose: Real-time visibility into PO activity, breaches, and operational priorities</t>
+  </si>
+  <si>
+    <t>8 KPIs for Procurement Dashboard</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>KPI name</t>
+  </si>
+  <si>
+    <t>What it answers (business question)</t>
+  </si>
+  <si>
+    <t>Total PO Value (MTD)</t>
+  </si>
+  <si>
+    <t>What's the total spend committed in POs this month?</t>
+  </si>
+  <si>
+    <t>SUM(02_PO_Dump.net_order_value) WHERE Creation_date BETWEEN month_start AND today AND deletion_indicator &lt;&gt; 'L'</t>
+  </si>
+  <si>
+    <t>Active PO Count</t>
+  </si>
+  <si>
+    <t>How many POs are currently Open?</t>
+  </si>
+  <si>
+    <t>COUNT(DISTINCT 02_PO_Dump.purchasing_document) WHERE delivery_completed &lt;&gt; 'X' AND deletion_indicator &lt;&gt; 'L'</t>
+  </si>
+  <si>
+    <t>High-Value PO Count</t>
+  </si>
+  <si>
+    <t>How many POs exceed the high-value threshold?</t>
+  </si>
+  <si>
+    <t>COUNT(DISTINCT 02_PO_Dump.purchasing_document) WHERE Realese_value &gt; [HIGH_VALUE_THRESHOLD] (default ₹1 Cr) AND deletion_indicator &lt;&gt; 'L'</t>
+  </si>
+  <si>
+    <t>Average PR-to-PO Conversion Time</t>
+  </si>
+  <si>
+    <t>How long does it take to convert a PR into a PO?</t>
+  </si>
+  <si>
+    <t>AVG(DATEDIFF(02_PO_Dump.Creation_date, 01_PR_Dump.Requisition_date)) WHERE 02_PO_Dump.purchase_requisition = 01_PR_Dump.purchase_requisition</t>
+  </si>
+  <si>
+    <t>PO Cycle Time (Creation → Approval)</t>
+  </si>
+  <si>
+    <t>How long does it take to get a PO approved?</t>
+  </si>
+  <si>
+    <t>AVG(DATEDIFF(release_date, creation_date)) FROM 02_PO_Dump WHERE release_indicator LIKE 'X%'</t>
+  </si>
+  <si>
+    <t>PO Deletion Frequency (MTD)</t>
+  </si>
+  <si>
+    <t>How many POs being deleted/cancelled in a month?</t>
+  </si>
+  <si>
+    <t>COUNT(02_PO_Dump.purchasing_document) WHERE deletion_indicator = 'L' AND document_date BETWEEN month_start AND today</t>
+  </si>
+  <si>
+    <t>PO Amendment Rate</t>
+  </si>
+  <si>
+    <t>What % of POs were modified after creation?</t>
+  </si>
+  <si>
+    <t>(COUNT(DISTINCT 09_Change_Log.object_id WHERE object_class='EINKBELEG') / COUNT(DISTINCT 02_PO_Dump.purchasing_document)) × 100</t>
+  </si>
+  <si>
+    <t>COUNT(01_PR_Dump.purchase_requisition) WHERE release_status='X' AND DATEDIFF(today, Creation_date) &gt; 7 AND purchase_requisition NOT IN (SELECT purchase_requisition FROM 02_PO_Dump)</t>
+  </si>
+  <si>
+    <t>Drill-down details (charts/tables on this dashboard)</t>
+  </si>
+  <si>
+    <t>• GM Trend Line Chart: KPI 1 plotted over last 12 months  • PO Status Bar: Active / Approved / Pending / Deleted counts per week  • High-Value PO Monitor Table: rows from 02_PO_Dump WHERE net_order_value &gt; threshold  • Compliance Alerts Card: links to KPI_04 vendor compliance breaches  • Upcoming Contract Renewals Card: 08_Vendor_Master JOIN contracts WHERE end_date &lt; today + 60 days</t>
+  </si>
+  <si>
+    <t>Formula Directions</t>
+  </si>
+  <si>
+    <t>Old Formula</t>
+  </si>
+  <si>
+    <t>New Formula</t>
+  </si>
+  <si>
+    <t>Change Instructions</t>
+  </si>
+  <si>
+    <t>SELECT SUM(CAST(net_order_value AS REAL))
+        FROM po_dump
+        WHERE (deletion_indicator IS NULL OR deletion_indicator NOT IN ('L','X'))
+          AND COALESCE(NULLIF(created_on,''), document_date) &gt;= {MTD}</t>
+  </si>
+  <si>
+    <t>SELECT COUNT(DISTINCT purchasing_document)
+        FROM po_dump
+        WHERE (deletion_indicator IS NULL OR deletion_indicator NOT IN ('L','X'))
+          AND (delivery_completed IS NULL OR delivery_completed = '')</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SELECT COUNT(DISTINCT purchasing_document)
+        FROM po_dump
+        WHERE (deletion_indicator IS NULL OR deletion_indicator NOT IN ('L','X'))
+          AND CAST(net_order_value AS REAL) &gt; {high_value_threshold}</t>
+  </si>
+  <si>
+    <t>SELECT AVG(CAST(min_po_days AS REAL))
+        FROM (
+            SELECT pr.purchase_requisition,
+                   pr.item_of_requisition,
+                   MIN(CAST(
+                       julianday(COALESCE(NULLIF(po.created_on,''), po.document_date))
+                       - julianday(COALESCE(NULLIF(pr.created_on,''), pr.release_date))
+                   AS INTEGER)) AS min_po_days
+            FROM pr_dump pr
+            JOIN po_dump po
+              ON po.purchase_requisition = pr.purchase_requisition
+             AND po.item_of_requisition  = pr.item_of_requisition
+            WHERE (po.deletion_indicator IS NULL OR po.deletion_indicator NOT IN ('L','X'))
+              AND COALESCE(NULLIF(pr.created_on,''), pr.release_date) IS NOT NULL
+              AND COALESCE(NULLIF(po.created_on,''), po.document_date) IS NOT NULL
+            GROUP BY pr.purchase_requisition, pr.item_of_requisition
+        )
+        WHERE min_po_days &gt;= 0</t>
+  </si>
+  <si>
+    <t>SELECT AVG(CAST(julianday(cl.change_date) - julianday(po.created_on) AS REAL))
+        FROM po_dump po #Remove Deleted POs from dump entirely
+        JOIN change_log cl
+          ON cl.object_id       = po.purchasing_document
+         AND cl.object_class    = 'EINKBELEG'
+         AND cl.field_name      IN ('FRGZU','FRGKE') #FRGKE is not important, could give unnecessary 
+         AND cl.change_indicator = 'U' #Could be E or U
+         AND cl.new_value        = 'X'
+        WHERE po.release_indicator = 'X' # Has to be Like X percentage, not X value
+          AND po.created_on IS NOT NULL AND po.created_on != ''</t>
+  </si>
+  <si>
+    <t>SELECT COUNT(DISTINCT purchasing_document) # With Append of Item Number, give info that PO Count is item level
+        FROM po_dump
+        WHERE deletion_indicator = 'L'
+          AND document_date &gt;= {MTD}</t>
+  </si>
+  <si>
+    <t>amended =&gt; 
+SELECT COUNT(DISTINCT cl.object_id)
+        FROM change_log cl
+        WHERE cl.object_class     = 'EINKBELEG'
+          AND cl.change_indicator  = 'U' 
+          AND cl.field_name NOT IN ('FRGZU', 'FRGKE', 'FRGRL', 'FRGGR')
+total =&gt;
+SELECT COUNT(DISTINCT purchasing_document) FROM po_dump
+        WHERE (deletion_indicator IS NULL OR deletion_indicator NOT IN ('L','X'))</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SELECT COUNT(DISTINCT pr.purchase_requisition || '|' || pr.item_of_requisition)
+        FROM pr_dump pr
+        WHERE pr.release_status IN ('X','XX','XXX','XXXX','XXXXX')
+          AND (pr.deletion_indicator IS NULL OR pr.deletion_indicator = '')
+          AND COALESCE(NULLIF(pr.created_on,''), pr.release_date) IS NOT NULL
+          AND julianday('{ref_date}') - julianday(COALESCE(NULLIF(pr.created_on,''), pr.release_date)) &gt; 7
+          AND NOT EXISTS (
+              SELECT 1 FROM po_dump po
+              WHERE po.purchase_requisition = pr.purchase_requisition
+                AND po.item_of_requisition  = pr.item_of_requisition
+                AND (po.deletion_indicator IS NULL OR po.deletion_indicator NOT IN ('L','X'))</t>
+  </si>
+  <si>
+    <t>Correct</t>
+  </si>
+  <si>
+    <t>Open PO Aging (&gt; 7 days)
+Changed from =&gt; Open PR Aging</t>
+  </si>
+  <si>
+    <t>How many POs are stuck without conversion?</t>
+  </si>
+  <si>
+    <t>Total PO Value (YTD)</t>
+  </si>
+  <si>
+    <t>PO Line Count (YTD)</t>
+  </si>
+  <si>
+    <t>SELECT SUM(CAST(net_order_value AS REAL))
+        FROM po_dump
+        WHERE (deletion_indicator IS NULL OR deletion_indicator NOT IN ('L','X'))
+          AND document_date &gt;= {FY}</t>
+  </si>
+  <si>
+    <t>SELECT COUNT(*) FROM po_dump
+        WHERE (deletion_indicator IS NULL OR deletion_indicator NOT IN ('L','X'))
+          AND document_date &gt;= {FY}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Step 1 — fact_builder.py (computes pr_to_po_days per item line)
+  SELECT
+      -- PR → PO days: PO.created_on (EKKO-ERDAT) minus PR.created_on (EBAN-ERDAT)
+      CASE WHEN pr.created_on IS NOT NULL AND pr.created_on != ''
+                AND po.created_on IS NOT NULL AND po.created_on != ''
+           THEN CAST(julianday(po.created_on) - julianday(pr.created_on) AS INTEGER)
+           ELSE NULL END AS pr_to_po_days
+  FROM po_dump po
+  LEFT JOIN pr_dump pr
+      ON po.company_code         = pr.company_code
+     AND po.purchase_requisition = pr.purchase_requisition
+     AND po.item_of_requisition  = pr.item_of_requisition
+  WHERE (po.deletion_indicator IS NULL OR po.deletion_indicator = '')
+    AND (pr.deletion_indicator  IS NULL OR pr.deletion_indicator != 'X')
+  GROUP BY po.purchasing_document, po.item
+  Step 2 — kpi_engine.py (aggregates into KPI card value)
+  SELECT AVG(CAST(pr_to_po_days AS REAL))
+  FROM pr_po_grn_invoice
+  WHERE pr_to_po_days     IS NOT NULL
+    AND pr_to_po_days     &gt;= 0
+    AND purchase_requisition IS NOT NULL
+    AND purchasing_document  IS NOT NULL
+  Flow: Upload → fact_builder joins PR+PO on 3 keys, stores day diff per line into pr_po_grn_invoice.pr_to_po_days →
+  kpi_engine reads fact table, averages → stored in kpi_results as PR_TO_PO_DAYS.</t>
+  </si>
+  <si>
+    <t>1. Join condition: PO Dump and PR Dump must be joined on three keys: Company Code, Purchase Requisition Number (EBAN-BANFN / EKPO-BANFN), and Item Number (EBAN-BNFPO / EKPO-BNFPO).
+2. Date calculation: Conversion time = PO Creation Date (EKKO-ERDAT) minus PR Requisition Date (EBAN-ERDAT). Average of this difference (in days) across all matched PR-PO item pairs is the KPI value.
+3. Deleted PR exclusion: PRs where Deletion Indicator (EBAN-LOEKZ) = 'X' must be excluded from the calculation. Only active (non-deleted) PRs are counted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  SELECT AVG(CAST(julianday(cl.change_date) - julianday(po.created_on) AS REAL))
+  FROM po_dump po
+  JOIN change_log cl
+    ON cl.object_id        = po.purchasing_document
+   AND cl.object_class     = 'EINKBELEG'
+   AND cl.field_name       = 'FRGZU'
+   AND cl.change_indicator IN ('E', 'U')
+   AND cl.new_value        LIKE 'X%'
+  WHERE po.release_indicator LIKE 'X%'
+    AND (po.deletion_indicator IS NULL OR po.deletion_indicator NOT IN ('L', 'X'))
+    AND po.created_on IS NOT NULL AND po.created_on != ''
+  Result stored in: kpi_results → kpi_code = 'PO_APPROVAL_CYCLE', unit = Days</t>
+  </si>
+  <si>
+    <t>1. Release Value Filter: changed from new_value='X' (only single-level approvals) to new_value LIKE 'X%' (captures all levels: X, XX, XXX). 
+2. Release Indicator Filter: changed from release_indicator='X' (excluded multi-level approvals) to release_indicator LIKE 'X%' (includes all released POs). 
+3. Change Indicator: extended from 'U' only (updates) to IN('E','U') (captures both first-time approvals 'E' and subsequent updates 'U'). 
+4. Field Name: narrowed from IN('FRGZU','FRGKE') to FRGZU only (FRGZU tracks release progression; FRGKE adds admin noise). 
+5. Deleted PO Exclusion: added deletion_indicator NOT IN('L','X') to exclude cancelled/abandoned POs; applied consistently across all KPI queries (P5, Maverick Spend Rate, Fact Table rebuild).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  KPI Card Value (kpi_results → PO_DELETION_MTD)
+  SELECT COUNT(DISTINCT purchasing_document || '|' || item)
+  FROM po_dump
+  WHERE deletion_indicator = 'L'
+    AND COALESCE(NULLIF(created_on, ''), document_date) &gt;= '&lt;MTD_START&gt;'
+  Monthly Trend (feeds bar chart via chart data API)
+  SELECT strftime('%Y-%m', COALESCE(NULLIF(created_on, ''), document_date)) AS month,
+         COUNT(DISTINCT purchasing_document || '|' || item)                  AS deleted_lines
+  FROM po_dump
+  WHERE deletion_indicator = 'L'
+    AND COALESCE(NULLIF(created_on, ''), document_date) &gt;= '&lt;12_MONTHS_AGO&gt;'
+  GROUP BY month</t>
+  </si>
+  <si>
+    <t>1. Date field changed from Document Date to Creation Date: previously used document_date (SAP BEDAT, can be backdated). Changed to COALESCE(NULLIF(created_on,''),document_date) where created_on=EKKO-ERDAT (system timestamp). This gives accurate creation timing for deletions; COALESCE handles blanks.
+2. Count granularity changed from Header level to Item level: deletion_indicator maps to EKPO-LOEKZ (item-level). A PO can have some items deleted and others active. Old method counted DISTINCT purchasing_document (undercounting). Changed to COUNT(DISTINCT purchasing_document || '|' || item) so each deleted line item is counted. Applies to P6 only; other KPIs remain header-level.
+3. Graphical display added (Bar Chart + KPI Card): P6 was computed and stored but not shown. Added KPI card in second row (danger indicator when count&gt;0) and monthly bar chart (PODeletionTrend) showing deletion trend by creation month over last 12 months. Existing detail table remains below.</t>
+  </si>
+  <si>
+    <t>1. Change Indicator: extended from 'U' only to IN('E','U'). SAP Change Log records E (initial entry, e.g. first material assignment) and U (update). Old filter only captured U, missing first-time entries. Now both included.
+2. Field Name: replaced broad exclusion with explicit inclusion of 4 business fields. Old logic used field_name NOT IN (release fields), which pulled in noise (user name, tcode, system fields). New strict positive list includes only: Material (EKPO-MATNR / MATNR), Net Order Price (EKPO-NETPR / NETPR), Net Order Value (EKPO-NETWR / NETWR), Quantity (EKPO-MENGE / MENGE).
+3. Join to PO Dump added (3-key logic). Old numerator queried change_log alone. Now joins on object_id = purchasing_document + company code (via po_dump). Item-level match uses CDPOS-TABKEY (last 5 chars = EBELP, leading zeros stripped): CAST(SUBSTR(table_key,-5) AS INTEGER) = CAST(po.item AS INTEGER). If table_key is NULL (not in CSV export), all items under that PO treated as amended. Full precision activates once TABKEY is included in export.
+4. Denominator changed to item level. Old: COUNT(DISTINCT purchasing_document) at header level. New: COUNT(DISTINCT purchasing_document || '|' || item) to match numerator grain. Rate now means: % of active PO line items with material/price/value/quantity change.
+5. table_key column added to schema. Added table_key TEXT column to change_log via migration-safe ALTER TABLE in database.py. Parser updated to accept it from CSV if present. Existing rows get NULL — no re-upload needed for other datasets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Numerator — Amended PO Line Items
+  SELECT COUNT(DISTINCT po.purchasing_document || '|' || po.item)
+  FROM po_dump po
+  JOIN change_log cl
+    ON  cl.object_id        = po.purchasing_document
+   AND  cl.object_class     = 'EINKBELEG'
+   AND  cl.change_indicator IN ('E', 'U')
+   AND  cl.field_name       IN ('MATNR', 'NETPR', 'NETWR', 'MENGE')
+   AND  (
+         cl.table_key IS NULL
+         OR cl.table_key = ''
+         OR CAST(SUBSTR(cl.table_key, -5) AS INTEGER) = CAST(po.item AS INTEGER)
+        )
+  WHERE (po.deletion_indicator IS NULL OR po.deletion_indicator NOT IN ('L', 'X'))
+  Denominator — Total Active PO Line Items
+  SELECT COUNT(DISTINCT purchasing_document || '|' || item)
+  FROM po_dump
+  WHERE (deletion_indicator IS NULL OR deletion_indicator NOT IN ('L', 'X'))
+  Rate
+  PO Amendment Rate (%) = (Numerator / Denominator) × 100</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,19 +348,142 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF00338D"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF757575"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF00338D"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF333333"/>
+      <name val="Consolas"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF333333"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF00338D"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00338D"/>
+        <bgColor rgb="FF333399"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5E9"/>
+        <bgColor rgb="FFF5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F5F5"/>
+        <bgColor rgb="FFE8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00A3A1"/>
+        <bgColor rgb="FF009FDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D1D1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D1D1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D1D1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D1D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D1D1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D1D1"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -49,8 +492,68 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +833,317 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="38" customWidth="1"/>
+    <col min="4" max="4" width="55" customWidth="1"/>
+    <col min="5" max="5" width="62.33203125" customWidth="1"/>
+    <col min="6" max="6" width="77.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="66.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="7"/>
+      <c r="G6" s="16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A7" s="8">
+        <v>2</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="7"/>
+      <c r="G7" s="17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="72" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
+        <v>3</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" s="7"/>
+      <c r="G8" s="16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="346.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="8">
+        <v>4</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="171" x14ac:dyDescent="0.3">
+      <c r="A10" s="5">
+        <v>5</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="204" x14ac:dyDescent="0.3">
+      <c r="A11" s="8">
+        <v>6</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="G11" s="20" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="286.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="5">
+        <v>7</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="G12" s="16" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="216" x14ac:dyDescent="0.3">
+      <c r="A13" s="8">
+        <v>8</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="7"/>
+      <c r="G13" s="14"/>
+    </row>
+    <row r="14" spans="1:7" ht="60" x14ac:dyDescent="0.3">
+      <c r="A14" s="8">
+        <v>9</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="19"/>
+      <c r="D14" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" s="15"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="48" x14ac:dyDescent="0.3">
+      <c r="A15" s="8">
+        <v>10</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="19"/>
+      <c r="D15" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="E15" s="15"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="10"/>
+    </row>
+    <row r="18" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+    </row>
+    <row r="19" spans="1:7" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A19:G19"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update IntelliSource Dashboard KPI Changes.xlsx
</commit_message>
<xml_diff>
--- a/IntelliSource Dashboard KPI Changes.xlsx
+++ b/IntelliSource Dashboard KPI Changes.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aryan\OneDrive\Documents\GitHub\kpmg-intelliflow\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAD905E0-6413-4F8A-8B6A-0B3327B09207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71E393DC-0A3E-4446-ACDD-0DA99B2EA946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Procurement Dashboard KPIs" sheetId="1" r:id="rId1"/>
+    <sheet name="Financial Dashboard KPIs" sheetId="3" r:id="rId1"/>
+    <sheet name="Procurement Dashboard KPIs" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="89">
   <si>
     <t>Procurement Dashboard — KPIs</t>
   </si>
@@ -334,6 +335,102 @@
   WHERE (deletion_indicator IS NULL OR deletion_indicator NOT IN ('L', 'X'))
   Rate
   PO Amendment Rate (%) = (Numerator / Denominator) × 100</t>
+  </si>
+  <si>
+    <t>Financial Dashboard — KPIs</t>
+  </si>
+  <si>
+    <t>Target user: Finance Team | Refresh: Monthly | Purpose: Spend vs budget tracking, cash flow, invoice/payment cycle health</t>
+  </si>
+  <si>
+    <t>8 KPIs for Financial Dashboard</t>
+  </si>
+  <si>
+    <t>Total Spend (YTD)</t>
+  </si>
+  <si>
+    <t>What's the total procurement spend this fiscal year?</t>
+  </si>
+  <si>
+    <t>07_Payment_Dump</t>
+  </si>
+  <si>
+    <t>Total amt of PO and Non PO invoices - cancelled Invoices , Doc Type - "RE" , "RN" , Non PO invoices - "KR" , Debit/Credit indicator - if "S" then refer amt *1 , else *-1 "h"</t>
+  </si>
+  <si>
+    <t>Cancellation Rate %</t>
+  </si>
+  <si>
+    <t>How much of the allocated budget have we consumed?</t>
+  </si>
+  <si>
+    <t>Cancelled Invoices / Total inv *100</t>
+  </si>
+  <si>
+    <t>Three-Way Match Success Rate (Can be removed)</t>
+  </si>
+  <si>
+    <t>What % of invoices match PO + GRN cleanly?</t>
+  </si>
+  <si>
+    <t>(COUNT(invoices WHERE 05_PO_Invoice_Dump.quantity = 04_GRN_Dump.quantity AND 05_PO_Invoice_Dump.amount_local_ccy ≈ 02_PO_Dump.net_order_value) / COUNT(05_PO_Invoice_Dump.invoice_doc)) × 100</t>
+  </si>
+  <si>
+    <t>02_PO_Dump + 04_GRN_Dump + 05_PO_Invoice_Dump</t>
+  </si>
+  <si>
+    <t>PO - PO line Items = SUM(GRN qty ) then True , (Take Cr/Db indicators into account for calculation th total GRN)</t>
+  </si>
+  <si>
+    <t>Invoice Processing Cycle Time</t>
+  </si>
+  <si>
+    <t>How long does it take to process an invoice?</t>
+  </si>
+  <si>
+    <t>AVG(DATEDIFF(06_Payement_Dump.clearing_date, 06_Invoice_Dump.vendor_invoice_date))</t>
+  </si>
+  <si>
+    <t>06_Invoice_Dump</t>
+  </si>
+  <si>
+    <t>Payment On-Time Rate</t>
+  </si>
+  <si>
+    <t>What % of invoices were paid on or before due date?</t>
+  </si>
+  <si>
+    <t>(COUNT(06_Invoice_Dump.invoice_doc WHERE clearing_doc IS NOT NULL AND 07_Payment_Dump.posting_date ≤ 06_Invoice_Dump.due_date) / COUNT(06_Invoice_Dump.invoice_doc WHERE clearing_doc IS NOT NULL)) × 100</t>
+  </si>
+  <si>
+    <t>06_Invoice_Dump + 07_Payment_Dump</t>
+  </si>
+  <si>
+    <t>Days Payable Outstanding (DPO)</t>
+  </si>
+  <si>
+    <t>On average how long do we take to pay vendors?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVG(DATEDIFF(07_Payment_Dump.posting_date, 06_Invoice_Dump.posting_date))  — for invoices linked to payments via clearing_doc </t>
+  </si>
+  <si>
+    <t>Open Invoice Aging (Total ₹)</t>
+  </si>
+  <si>
+    <t>How much do we owe vendors in unpaid invoices?</t>
+  </si>
+  <si>
+    <t>(06_Invoice_Dump.posting_date) WHERE clearing_doc IS NULL  — bucketed by 0-30 / 31-60 / 61-90 / 90+ days from posting_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Early / Delayed Payment count </t>
+  </si>
+  <si>
+    <t>Invoice Before due date , after due date</t>
+  </si>
+  <si>
+    <t>Change Directions</t>
   </si>
 </sst>
 </file>
@@ -454,7 +551,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -488,11 +585,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD1D1D1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D1D1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D1D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D1D1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D1D1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD1D1D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD1D1D1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD1D1D1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -524,35 +658,62 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -833,6 +994,236 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC8E4E0-1D19-4614-B875-28C220820B5F}">
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="38" customWidth="1"/>
+    <col min="4" max="6" width="65" customWidth="1"/>
+    <col min="7" max="7" width="32.109375" customWidth="1"/>
+    <col min="8" max="8" width="63.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A1" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="24" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D6" s="25"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6" s="27" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="8">
+        <v>2</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="D7" s="25"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="28"/>
+      <c r="H7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="48.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
+        <v>3</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="H8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="24.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="8">
+        <v>4</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="28" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="48.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="5">
+        <v>5</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="26" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="36.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="8">
+        <v>6</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="28" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="24.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="5">
+        <v>7</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="26" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="8">
+        <v>8</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="28" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A4:D4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G19"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -847,38 +1238,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
     </row>
     <row r="2" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
     </row>
     <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
     </row>
     <row r="5" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
@@ -899,7 +1290,7 @@
       <c r="F5" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="11" t="s">
         <v>33</v>
       </c>
     </row>
@@ -916,11 +1307,11 @@
       <c r="D6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="13" t="s">
         <v>34</v>
       </c>
       <c r="F6" s="7"/>
-      <c r="G6" s="16" t="s">
+      <c r="G6" s="14" t="s">
         <v>42</v>
       </c>
     </row>
@@ -937,11 +1328,11 @@
       <c r="D7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="15" t="s">
+      <c r="E7" s="13" t="s">
         <v>35</v>
       </c>
       <c r="F7" s="7"/>
-      <c r="G7" s="17" t="s">
+      <c r="G7" s="15" t="s">
         <v>42</v>
       </c>
     </row>
@@ -958,11 +1349,11 @@
       <c r="D8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="E8" s="13" t="s">
         <v>36</v>
       </c>
       <c r="F8" s="7"/>
-      <c r="G8" s="16" t="s">
+      <c r="G8" s="14" t="s">
         <v>42</v>
       </c>
     </row>
@@ -979,13 +1370,13 @@
       <c r="D9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="15" t="s">
+      <c r="E9" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="G9" s="17" t="s">
+      <c r="G9" s="15" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1002,13 +1393,13 @@
       <c r="D10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="E10" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="G10" s="16" t="s">
+      <c r="G10" s="14" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1025,13 +1416,13 @@
       <c r="D11" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="G11" s="18" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1048,13 +1439,13 @@
       <c r="D12" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="G12" s="16" t="s">
+      <c r="G12" s="14" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1062,35 +1453,35 @@
       <c r="A13" s="8">
         <v>8</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="17" t="s">
         <v>44</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="15" t="s">
+      <c r="E13" s="13" t="s">
         <v>41</v>
       </c>
       <c r="F13" s="7"/>
-      <c r="G13" s="14"/>
+      <c r="G13" s="12"/>
     </row>
     <row r="14" spans="1:7" ht="60" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>9</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="15" t="s">
+      <c r="C14" s="17"/>
+      <c r="D14" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="E14" s="15"/>
+      <c r="E14" s="13"/>
       <c r="F14" s="7"/>
-      <c r="G14" s="17" t="s">
+      <c r="G14" s="15" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1098,16 +1489,16 @@
       <c r="A15" s="8">
         <v>10</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="15" t="s">
+      <c r="C15" s="17"/>
+      <c r="D15" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="E15" s="15"/>
+      <c r="E15" s="13"/>
       <c r="F15" s="7"/>
-      <c r="G15" s="17" t="s">
+      <c r="G15" s="15" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1115,26 +1506,26 @@
       <c r="A16" s="10"/>
     </row>
     <row r="18" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
     </row>
     <row r="19" spans="1:7" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>